<commit_message>
Fixed ART-DECOR-id link, added pagecontents
</commit_message>
<xml_diff>
--- a/input/requirements/Location.xlsx
+++ b/input/requirements/Location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Location/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="263" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02AD06A-5AEC-4349-B6EA-1F537358EED3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B00F28-2FD2-4742-ABAE-5DF9D7046F1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="5" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-2280" yWindow="-27080" windowWidth="34560" windowHeight="21660" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>ART-DECOR-id</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.4.3.11.60.153.1.8</t>
-  </si>
-  <si>
     <t>Nummer</t>
   </si>
   <si>
@@ -277,13 +274,16 @@
   </si>
   <si>
     <t>Onduidelijk welke informatie hiermee bedoeld wordt in de zib, omdat het al wordt gedekt door het Organization profiel.</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.22/2026-06-25T00:00:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1583,12 +1583,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="218.42578125" customWidth="1"/>
+    <col min="1" max="1" width="218.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
   </sheetData>
@@ -1600,16 +1600,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="108.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="108.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="190.5" customHeight="1">
+    <row r="1" spans="1:2" ht="190.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45">
+    <row r="3" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="231">
+    <row r="8" spans="1:2" ht="256" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="66.75" customHeight="1">
+    <row r="9" spans="1:2" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1673,17 +1673,17 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1695,197 +1695,197 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" customWidth="1"/>
-    <col min="3" max="3" width="68.42578125" customWidth="1"/>
-    <col min="4" max="4" width="63.85546875" customWidth="1"/>
-    <col min="5" max="6" width="48.7109375" customWidth="1"/>
-    <col min="7" max="7" width="52.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="68.5" customWidth="1"/>
+    <col min="4" max="4" width="63.83203125" customWidth="1"/>
+    <col min="5" max="6" width="48.6640625" customWidth="1"/>
+    <col min="7" max="7" width="52.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="191.25" customHeight="1"/>
-    <row r="2" spans="1:7">
+    <row r="1" spans="1:7" ht="191.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" s="3" customFormat="1">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" s="3" customFormat="1">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="G5" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="3" customFormat="1" ht="29.25">
-      <c r="A6" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" ht="29.25">
-      <c r="A7" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="3" customFormat="1">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="3" t="s">
+    </row>
+    <row r="9" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" s="3" customFormat="1">
-      <c r="A9" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="3" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A10" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="3" customFormat="1">
-      <c r="A11" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="D11" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1899,60 +1899,60 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1964,9 +1964,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" ht="111" customHeight="1"/>
+    <row r="1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1976,18 +1976,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F35EFE-AF73-4557-BEE4-B434F85A1F85}">
   <dimension ref="A2:I21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="19.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="77.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="76.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="77.5" style="3" customWidth="1"/>
+    <col min="5" max="5" width="76.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5"/>
       <c r="B2" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -1997,35 +1997,35 @@
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
       <c r="I3" s="5"/>
     </row>
-    <row r="4" spans="1:9" ht="29.25">
+    <row r="4" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>73</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="5"/>
@@ -2033,103 +2033,103 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
     </row>
-    <row r="20" spans="2:5">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
     </row>
-    <row r="21" spans="2:5">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
@@ -2144,15 +2144,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -2161,6 +2152,15 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2371,13 +2371,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Remove example row in Informatiebehoefte tab
</commit_message>
<xml_diff>
--- a/input/requirements/Location.xlsx
+++ b/input/requirements/Location.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B00F28-2FD2-4742-ABAE-5DF9D7046F1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5DFAB3-2FD0-5A4B-BA34-2D59EDF12FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2280" yWindow="-27080" windowWidth="34560" windowHeight="21660" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" firstSheet="1" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
   <si>
     <t>Veld</t>
   </si>
@@ -128,12 +128,6 @@
     <t>Herkomst</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
-  </si>
-  <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
   </si>
   <si>
@@ -141,9 +135,6 @@
   </si>
   <si>
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
   </si>
   <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
@@ -1683,7 +1674,7 @@
         <v>16</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1694,7 +1685,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
@@ -1729,61 +1720,55 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="1" t="s">
+    <row r="3" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>30</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>39</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
@@ -1797,47 +1782,47 @@
         <v>42</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>51</v>
       </c>
@@ -1848,13 +1833,13 @@
         <v>53</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>54</v>
       </c>
@@ -1865,27 +1850,10 @@
         <v>56</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1911,10 +1879,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>18</v>
@@ -1934,25 +1902,25 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1987,7 +1955,7 @@
     <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5"/>
       <c r="B2" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -2000,16 +1968,16 @@
     <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>66</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>69</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
@@ -2019,13 +1987,13 @@
     <row r="4" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="5"/>
@@ -2144,6 +2112,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -2152,15 +2129,6 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2371,20 +2339,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
     <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Location: refreshed requirements file
</commit_message>
<xml_diff>
--- a/input/requirements/Location.xlsx
+++ b/input/requirements/Location.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Location/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="263" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02AD06A-5AEC-4349-B6EA-1F537358EED3}"/>
+  <xr:revisionPtr revIDLastSave="401" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9BB2102-06C7-49CD-A179-3E59B7845D08}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="5" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
     <sheet name="Concept" sheetId="2" r:id="rId2"/>
-    <sheet name="Informatiebehoefte" sheetId="1" r:id="rId3"/>
-    <sheet name="Ongedekte informatiebehoefte" sheetId="3" r:id="rId4"/>
-    <sheet name="Overwegingen voor de toekomst" sheetId="4" r:id="rId5"/>
-    <sheet name="Ter Discussie" sheetId="6" r:id="rId6"/>
+    <sheet name="Bronnen" sheetId="7" r:id="rId3"/>
+    <sheet name="Informatiebehoefte" sheetId="1" r:id="rId4"/>
+    <sheet name="Ongedekte informatiebehoefte" sheetId="3" r:id="rId5"/>
+    <sheet name="Overwegingen voor de toekomst" sheetId="4" r:id="rId6"/>
+    <sheet name="Ter Discussie" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
   <si>
     <t>Veld</t>
   </si>
@@ -52,7 +53,7 @@
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>A Location includes both incidental locations (a place which is used for healthcare without prior designation or authorization) and dedicated, formally appointed locations. Locations may be private, public, mobile or fixed and scale from small freezers to full hospital buildings or parking garages.</t>
+    <t>Een locatie omvat zowel incidentele locaties (een plek die zonder voorafgaande aanwijzing of toestemming voor gezondheidszorg wordt gebruikt) als speciale, formeel aangewezen locaties. Locaties kunnen particulier, openbaar, mobiel of vast zijn en variëren in omvang van kleine vrieskisten tot complete ziekenhuisgebouwen of parkeergarages.</t>
   </si>
   <si>
     <t>Doel</t>
@@ -79,35 +80,103 @@
     <t>Juist gebruik</t>
   </si>
   <si>
-    <t>Physical location
- A Location includes both incidental locations (a place which is used for healthcare without prior designation or authorization) and dedicated, formally appointed locations. Locations may be private, public, mobile or fixed and scale from small freezers to full hospital buildings or parking garages.
-Examples of Locations are:
-Building, ward, corridor, room or bed
-Mobile Clinic
-Freezer, incubator
-Vehicle or lift
-Home, shed, or a garage
-Road, parking place, a park
-Ambulance (generic)
-Ambulance (specific)
-Patient's Home (generic)
-Jurisdiction</t>
+    <t>Een fysieke locatie
+Voorbeelden van locaties zijn:
+Gebouw, afdeling, gang, kamer of bed
+Mobiele kliniek
+Vriezer, couveuse
+Voertuig of lift
+Huis, schuur of garage
+Weg, parkeerplaats, park
+Ambulance (algemeen)
+Ambulance (specifiek)
+Huis van de patiënt (algemeen)
+Rechtsgebied</t>
   </si>
   <si>
     <t>Onjuist gebruik</t>
   </si>
   <si>
-    <t>Location is a physical place, and should not be used to represent conceptual hierarchies such as a ward.
-Location should not be used to cover locations on a patient where something occurred (i.e. a patient's broken leg), but can happily cover the location where the patient broke the leg (the playground).</t>
+    <t>Een locatie is een fysieke plek en mag niet worden gebruikt om conceptuele hiërarchieën weer te geven, zoals een ziekenhuisafdeling.
+Een locatie mag niet worden gebruikt om plaatsen op het lichaam van een patiënt aan te duiden waar iets is gebeurd (bijvoorbeeld een gebroken been van een patiënt), maar kan wel degelijk de locatie aangeven waar de patiënt zijn been heeft gebroken (de speelplaats).</t>
   </si>
   <si>
     <t>Referenties</t>
   </si>
   <si>
+    <t>Zie tabblad Bronnen</t>
+  </si>
+  <si>
     <t>ART-DECOR-id</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.4.3.11.60.153.1.8</t>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.22/2026-06-25T00:00:00</t>
+  </si>
+  <si>
+    <t>type bron</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>aantekeningen</t>
+  </si>
+  <si>
+    <t>zibs.nl</t>
+  </si>
+  <si>
+    <t>https://zibs.nl/wiki/Zorgaanbieder-v3.4(2020NL)</t>
+  </si>
+  <si>
+    <t>openEHR</t>
+  </si>
+  <si>
+    <t>https://ckm.openehr.org/ckm/archetypes/1013.1.5742/mindmap</t>
+  </si>
+  <si>
+    <t>GeoLocation</t>
+  </si>
+  <si>
+    <t>FHIR R4 base</t>
+  </si>
+  <si>
+    <t>https://hl7.org/fhir/R4/location.html</t>
+  </si>
+  <si>
+    <t>zib-profiel</t>
+  </si>
+  <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/zibhealthcareprovider</t>
+  </si>
+  <si>
+    <t>NL-core-R4</t>
+  </si>
+  <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/nlcorehealthcareprovider</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM</t>
+  </si>
+  <si>
+    <t>https://build.fhir.org/ig/Xt-EHR/xt-ehr-common/en/StructureDefinition-EHDSLocation.html</t>
+  </si>
+  <si>
+    <t>EHDS FHIR</t>
+  </si>
+  <si>
+    <t>https://hl7.eu/fhir/base/StructureDefinition-location-eu-core.html</t>
+  </si>
+  <si>
+    <t>mapping xt-EHR --&gt; FHIR</t>
+  </si>
+  <si>
+    <t>https://hl7.eu/fhir/base/map-ehdslocation.html</t>
+  </si>
+  <si>
+    <t>zib-issues</t>
+  </si>
+  <si>
+    <t>Speodsamenvatting</t>
   </si>
   <si>
     <t>Nummer</t>
@@ -131,25 +200,7 @@
     <t>Herkomst</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
-  </si>
-  <si>
-    <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
-  </si>
-  <si>
-    <t>[Geef aan wat het element waarmee de informatie-requirement gedekt wordt allemaal zou moeten kunnen. Is het bv. een exacte tijd, en/of een datum, en/of een seizoen?]</t>
-  </si>
-  <si>
-    <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
-  </si>
-  <si>
-    <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
+    <t>Opmerkingen</t>
   </si>
   <si>
     <t>LOC-001</t>
@@ -161,10 +212,13 @@
     <t>Location identifier</t>
   </si>
   <si>
+    <t>(identifier)</t>
+  </si>
+  <si>
     <t>0..*</t>
   </si>
   <si>
-    <t>Xt-EHR LIM 1.0.0 Location</t>
+    <t>EHDSLocation</t>
   </si>
   <si>
     <t>LOC-002</t>
@@ -176,9 +230,15 @@
     <t>Name of the location as used by humans</t>
   </si>
   <si>
+    <t>(string)</t>
+  </si>
+  <si>
     <t>0..1</t>
   </si>
   <si>
+    <t>EHDSLocation, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
     <t>LOC-003</t>
   </si>
   <si>
@@ -197,62 +257,68 @@
     <t>Type of function performed at the location</t>
   </si>
   <si>
-    <t>0..*
+    <t>(code)
 Binding Description: (preferred): HL7 ServiceDeliveryLocationRoleType</t>
   </si>
   <si>
     <t>LOC-005</t>
   </si>
   <si>
-    <t>Telecom</t>
-  </si>
-  <si>
-    <t>Contact details of the location</t>
-  </si>
-  <si>
-    <t>zib2020 HealthProvider</t>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Physical location</t>
+  </si>
+  <si>
+    <t>(ref. GBB-Address)</t>
   </si>
   <si>
     <t>LOC-006</t>
   </si>
   <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Physical location</t>
+    <t>ManagingOrganization</t>
+  </si>
+  <si>
+    <t>Organization responsible for provisioning and upkeep of the location</t>
+  </si>
+  <si>
+    <t>(ref. GBB-Organization)</t>
   </si>
   <si>
     <t>LOC-007</t>
   </si>
   <si>
-    <t>ManagingOrganization</t>
-  </si>
-  <si>
-    <t>Organization responsible for provisioning and upkeep of the location</t>
-  </si>
-  <si>
-    <t>LOC-008</t>
-  </si>
-  <si>
     <t>PartOf</t>
   </si>
   <si>
     <t>Another location of which this location is physically a part of</t>
   </si>
   <si>
+    <t>(ref. GBB-Location)</t>
+  </si>
+  <si>
+    <t>0..1  If the resource is contained in another resource, it SHALL NOT contain nested Resources. e.g., a department in a hospital cannot be the target of another Location.partOf</t>
+  </si>
+  <si>
     <t>Actie</t>
   </si>
   <si>
     <t>Notitie</t>
   </si>
   <si>
-    <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
-  </si>
-  <si>
-    <t>[Eventuele notitie]</t>
-  </si>
-  <si>
-    <t>[Naam van de informatie-requirement ]</t>
+    <t>Vraag aan leveranciers of ze dit FHIR-profiel willen gebruiken</t>
+  </si>
+  <si>
+    <t>Dit is een erg belangrijk concept als het gaat om PractitionerRole, Organization en Location: het geeft aan wat een organisatie doet voor een Patient in een bepaalde locatie (bijv. een departement of apotheek).</t>
+  </si>
+  <si>
+    <t>HealthCareService FHIR-resource</t>
+  </si>
+  <si>
+    <t>Komt noch in EHDSLocation als zib2020 voor, maar bepaalde Locaties kunnen wel specifieke contactgegevens hebben</t>
+  </si>
+  <si>
+    <t>telecom</t>
   </si>
   <si>
     <t>Ter Discussie</t>
@@ -277,13 +343,25 @@
   </si>
   <si>
     <t>Onduidelijk welke informatie hiermee bedoeld wordt in de zib, omdat het al wordt gedekt door het Organization profiel.</t>
+  </si>
+  <si>
+    <t>Verwijderen voor nu (zie overwegingen voor de toekomst)</t>
+  </si>
+  <si>
+    <t>LocationNumber</t>
+  </si>
+  <si>
+    <t>nlcore comment op HealthcareProvider : "In consultation with 'Registratie aan de Bron', it is agreed to not include the zib concept LocationNumber (NL-CM:17.2.10) due to several reasons. Firstly, its use in the Dutch realm is unclear as this concept was initiated for the Belgium realm with specific requirements. Secondly, it cannot be mapped neatly in the FHIR model which would require the use of an extension. To avoid implementation of specific and not-used FHIR requirements, it is advised to create and use an extension at the use case level where this concept is deemed necessary."</t>
+  </si>
+  <si>
+    <t>LocationNumber is geen Identifier. Niet opgenomen als IB.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,14 +371,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -343,13 +413,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE97132"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -372,18 +469,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -391,26 +494,42 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="39">
     <dxf>
       <font>
         <b val="0"/>
@@ -544,6 +663,188 @@
         </patternFill>
       </fill>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FFE97132"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1175,13 +1476,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>85725</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>100011</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>561975</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1266824</xdr:rowOff>
+      <xdr:rowOff>1266825</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1196,8 +1497,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="85725" y="100011"/>
-          <a:ext cx="5353050" cy="1166813"/>
+          <a:off x="85725" y="95250"/>
+          <a:ext cx="5286375" cy="1171575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1253,6 +1554,78 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC4B3689-B5E1-4C0B-8A18-2EF6796FA910}" name="Tabel2" displayName="Tabel2" ref="A2:B11" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+  <autoFilter ref="A2:B11" xr:uid="{BC4B3689-B5E1-4C0B-8A18-2EF6796FA910}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{19A2441A-EF17-41BD-B7AE-2B44CB1390B2}" name="Veld" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{0EFCC567-0804-4A16-B4C6-ECB35713CFDF}" name="Beschrijving" dataDxfId="35"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0FBA59BE-FED1-4830-9B47-92B0E9986636}" name="Tabel3" displayName="Tabel3" ref="A1:C12" totalsRowShown="0" headerRowDxfId="34">
+  <autoFilter ref="A1:C12" xr:uid="{0FBA59BE-FED1-4830-9B47-92B0E9986636}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{6D7BA7AB-73CA-4A29-88BB-60C2AD2B18E4}" name="type bron" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{62FCCC29-45BD-407A-B728-9557840FE3DB}" name="link"/>
+    <tableColumn id="3" xr3:uid="{EA8EAFC8-B0BA-405D-9518-EB07527142ED}" name="aantekeningen"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}" name="Tabel5" displayName="Tabel5" ref="A2:H9" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+  <autoFilter ref="A2:H9" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{853B139C-8A9D-42FA-A1DE-FF181BA77A00}" name="Nummer" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{700EFCE4-2DD7-46D2-8B8A-C706634BCB30}" name="Naam" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{2D7A676C-261C-4CA2-9EE7-2C4DFE8E8BC9}" name="Omschrijving" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{3A92D932-0952-474C-901F-7081BB4B3EEB}" name="Variabiliteit" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{63133D85-A35B-4E57-A2B1-1FC8C3320954}" name="Aanwezigheid"/>
+    <tableColumn id="6" xr3:uid="{D55E3300-913F-4340-8FAD-64BB21FB6FC0}" name="Verleden/heden/toekomst" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{C3BD8C6A-D06A-4FB0-BCA1-5C03A6EC7055}" name="Herkomst" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{80C27CD6-7638-4FAB-8D19-DA2D456BCFFB}" name="Opmerkingen" dataDxfId="24"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{9588B8FC-3CB6-466F-B8B0-B6E358CE159F}" name="Tabel8" displayName="Tabel8" ref="A1:G2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="A1:G2" xr:uid="{9588B8FC-3CB6-466F-B8B0-B6E358CE159F}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{2C39DF8A-8FD6-4530-AABD-23C9F73FF0CA}" name="Actie" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{0351DEEB-DAAB-48F0-BAD5-9C2CDFB46E9B}" name="Notitie" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{CEEBCE0E-57D3-459B-9F36-78A5E6DB6AE7}" name="Naam" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{4EB1F421-49CF-426F-9C52-A988A5438887}" name="Omschrijving" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{2590127D-AC2B-42F0-89BB-0908E1C8B4FC}" name="Variabiliteit" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{CF358206-3929-48A8-8B66-A9AA5FE44187}" name="Aanwezigheid" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{50C40459-B344-4551-AFE9-1D6674259227}" name="Herkomst" dataDxfId="15"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B070721D-114A-439E-9C4D-B340A09CA051}" name="Tabel810" displayName="Tabel810" ref="A2:G3" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+  <autoFilter ref="A2:G3" xr:uid="{B070721D-114A-439E-9C4D-B340A09CA051}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{A859077D-E5DB-43FC-A6F7-9ACAC1C2A3CE}" name="Actie" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{C875C01C-3FC3-46C2-A377-F5EB33F51C1E}" name="Notitie" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{56E92CFD-FB03-44C5-ACE9-14D49EAD629E}" name="Naam" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{12B3AC5B-FA22-4232-AD89-BC4BFDC87625}" name="Omschrijving" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{4239A765-C3A8-4EE0-BDFA-899815CDE3BB}" name="Variabiliteit" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{FCFF7AA3-4AF4-4A63-BC2E-A9927E9138A4}" name="Aanwezigheid" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{1D73E3B6-45A6-4810-BD8A-8CD9AB607D5B}" name="Herkomst" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0B0D1EB-FBDD-403B-B84C-855C7FFB0C48}" name="Tabel1" displayName="Tabel1" ref="B3:E21" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="B3:E21" xr:uid="{B0B0D1EB-FBDD-403B-B84C-855C7FFB0C48}"/>
   <tableColumns count="4">
@@ -1583,13 +1956,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="218.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15" customHeight="1">
-      <c r="A1" s="3"/>
+      <c r="A1" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1602,100 +1975,223 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="108.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="23" style="15" customWidth="1"/>
+    <col min="2" max="2" width="136.140625" style="14" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="190.5" customHeight="1">
-      <c r="A1" s="3"/>
+      <c r="A1" s="14"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2" ht="43.5">
+      <c r="A3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="A4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="14" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="A5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s">
+      <c r="A6" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" t="s">
+      <c r="A7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="231">
-      <c r="A8" t="s">
+    <row r="8" spans="1:2" ht="200.25" customHeight="1">
+      <c r="A8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="66.75" customHeight="1">
-      <c r="A9" t="s">
+    <row r="9" spans="1:2" ht="51.75" customHeight="1">
+      <c r="A9" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" t="s">
+      <c r="A10" s="15" t="s">
         <v>15</v>
       </c>
+      <c r="B10" s="14" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="A11" s="15" t="s">
         <v>17</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5848A0C1-D9F1-4267-9563-93913EA9663E}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="80.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="29.1">
+      <c r="A4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="29.1">
+      <c r="A5" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="29.25">
+      <c r="A6" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="29.1">
+      <c r="A7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="29.1">
+      <c r="A8" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="43.5">
+      <c r="A9" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="29.1">
+      <c r="A10" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="12"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{CFAB93B3-2904-468F-A314-3F5F787120D6}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{9467FB35-9215-47B0-B560-3C502EA216C6}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{BE147878-009C-400F-B2F7-690D8B78CF40}"/>
+    <hyperlink ref="B8" r:id="rId4" xr:uid="{76D68913-B017-4AD6-B5D2-D650B055D0FC}"/>
+    <hyperlink ref="B9" r:id="rId5" xr:uid="{F3C1C080-F118-4D40-A5A4-13FE67473D97}"/>
+    <hyperlink ref="B4" r:id="rId6" xr:uid="{3A4FBCE2-8F3F-4981-AB53-893FB24C62E2}"/>
+    <hyperlink ref="B5" r:id="rId7" xr:uid="{71EB33F5-B15F-4B62-97D9-38E24134FB0F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId8"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
     <col min="2" max="2" width="27.7109375" customWidth="1"/>
@@ -1703,206 +2199,195 @@
     <col min="4" max="4" width="63.85546875" customWidth="1"/>
     <col min="5" max="6" width="48.7109375" customWidth="1"/>
     <col min="7" max="7" width="52.85546875" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="191.25" customHeight="1"/>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="3" customFormat="1">
-      <c r="A4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="3" customFormat="1">
-      <c r="A5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="3" customFormat="1" ht="29.25">
-      <c r="A6" s="3" t="s">
+    <row r="1" spans="1:8" ht="191.25" customHeight="1"/>
+    <row r="2" spans="1:8" ht="15">
+      <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" ht="29.25">
-      <c r="A7" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="3" customFormat="1">
-      <c r="A8" s="3" t="s">
+      <c r="H2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="3" t="s">
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" ht="15">
+      <c r="A3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" s="3" customFormat="1">
-      <c r="A9" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="E3" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="3" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A10" s="3" t="s">
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" ht="15">
+      <c r="A4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="3" customFormat="1">
-      <c r="A11" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="E4" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>36</v>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="29.25">
+      <c r="A5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="29.25">
+      <c r="A6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="15">
+      <c r="A7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="20.25" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="2" customFormat="1" ht="57.75">
+      <c r="A9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.42578125" customWidth="1"/>
     <col min="4" max="4" width="15.140625" customWidth="1"/>
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
@@ -1910,230 +2395,281 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
+      <c r="A1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" ht="80.25" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" ht="111" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="15"/>
+    <col min="2" max="2" width="52.5703125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="15"/>
+    <col min="4" max="4" width="32" style="15" customWidth="1"/>
+    <col min="5" max="5" width="23" style="15" customWidth="1"/>
+    <col min="6" max="6" width="24.140625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="23" style="15" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="111" customHeight="1"/>
+    <row r="2" spans="1:7" s="16" customFormat="1">
+      <c r="A2" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="29.25">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F35EFE-AF73-4557-BEE4-B434F85A1F85}">
   <dimension ref="A2:I21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="19.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="77.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="76.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="77.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="76.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="5"/>
-      <c r="B3" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="4" spans="1:9" ht="29.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="29.1">
+      <c r="A4" s="3"/>
+      <c r="B4" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="101.45">
+      <c r="B5" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
     <row r="17" spans="2:5">
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
     </row>
     <row r="18" spans="2:5">
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
     </row>
     <row r="20" spans="2:5">
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2153,17 +2689,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -2370,14 +2895,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
 </file>
</xml_diff>

<commit_message>
Location: added EU filter row
</commit_message>
<xml_diff>
--- a/input/requirements/Location.xlsx
+++ b/input/requirements/Location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Location/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="401" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9BB2102-06C7-49CD-A179-3E59B7845D08}"/>
+  <xr:revisionPtr revIDLastSave="402" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3781AAC8-A544-411A-AB1E-FFC3E9FF8ED9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="101">
   <si>
     <t>Veld</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>Opmerkingen</t>
+  </si>
+  <si>
+    <t>EU filter</t>
   </si>
   <si>
     <t>LOC-001</t>
@@ -435,7 +438,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -448,8 +451,20 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -468,12 +483,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -521,15 +549,21 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
+  <dxfs count="40">
     <dxf>
       <font>
         <b val="0"/>
@@ -748,6 +782,10 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1554,21 +1592,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC4B3689-B5E1-4C0B-8A18-2EF6796FA910}" name="Tabel2" displayName="Tabel2" ref="A2:B11" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC4B3689-B5E1-4C0B-8A18-2EF6796FA910}" name="Tabel2" displayName="Tabel2" ref="A2:B11" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A2:B11" xr:uid="{BC4B3689-B5E1-4C0B-8A18-2EF6796FA910}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{19A2441A-EF17-41BD-B7AE-2B44CB1390B2}" name="Veld" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{0EFCC567-0804-4A16-B4C6-ECB35713CFDF}" name="Beschrijving" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{19A2441A-EF17-41BD-B7AE-2B44CB1390B2}" name="Veld" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{0EFCC567-0804-4A16-B4C6-ECB35713CFDF}" name="Beschrijving" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0FBA59BE-FED1-4830-9B47-92B0E9986636}" name="Tabel3" displayName="Tabel3" ref="A1:C12" totalsRowShown="0" headerRowDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0FBA59BE-FED1-4830-9B47-92B0E9986636}" name="Tabel3" displayName="Tabel3" ref="A1:C12" totalsRowShown="0" headerRowDxfId="35">
   <autoFilter ref="A1:C12" xr:uid="{0FBA59BE-FED1-4830-9B47-92B0E9986636}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6D7BA7AB-73CA-4A29-88BB-60C2AD2B18E4}" name="type bron" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{6D7BA7AB-73CA-4A29-88BB-60C2AD2B18E4}" name="type bron" dataDxfId="34"/>
     <tableColumn id="2" xr3:uid="{62FCCC29-45BD-407A-B728-9557840FE3DB}" name="link"/>
     <tableColumn id="3" xr3:uid="{EA8EAFC8-B0BA-405D-9518-EB07527142ED}" name="aantekeningen"/>
   </tableColumns>
@@ -1577,17 +1615,20 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}" name="Tabel5" displayName="Tabel5" ref="A2:H9" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
-  <autoFilter ref="A2:H9" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{853B139C-8A9D-42FA-A1DE-FF181BA77A00}" name="Nummer" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{700EFCE4-2DD7-46D2-8B8A-C706634BCB30}" name="Naam" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{2D7A676C-261C-4CA2-9EE7-2C4DFE8E8BC9}" name="Omschrijving" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{3A92D932-0952-474C-901F-7081BB4B3EEB}" name="Variabiliteit" dataDxfId="27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}" name="Tabel5" displayName="Tabel5" ref="A2:I9" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+  <autoFilter ref="A2:I9" xr:uid="{409C3BE5-F7AF-4DF5-8804-3FD022E318D0}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{853B139C-8A9D-42FA-A1DE-FF181BA77A00}" name="Nummer" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{700EFCE4-2DD7-46D2-8B8A-C706634BCB30}" name="Naam" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{2D7A676C-261C-4CA2-9EE7-2C4DFE8E8BC9}" name="Omschrijving" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{3A92D932-0952-474C-901F-7081BB4B3EEB}" name="Variabiliteit" dataDxfId="28"/>
     <tableColumn id="5" xr3:uid="{63133D85-A35B-4E57-A2B1-1FC8C3320954}" name="Aanwezigheid"/>
-    <tableColumn id="6" xr3:uid="{D55E3300-913F-4340-8FAD-64BB21FB6FC0}" name="Verleden/heden/toekomst" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{C3BD8C6A-D06A-4FB0-BCA1-5C03A6EC7055}" name="Herkomst" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{80C27CD6-7638-4FAB-8D19-DA2D456BCFFB}" name="Opmerkingen" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{D55E3300-913F-4340-8FAD-64BB21FB6FC0}" name="Verleden/heden/toekomst" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{C3BD8C6A-D06A-4FB0-BCA1-5C03A6EC7055}" name="Herkomst" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{80C27CD6-7638-4FAB-8D19-DA2D456BCFFB}" name="Opmerkingen" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{4C2B8F99-4657-474A-9896-251F99DD789A}" name="EU filter" dataDxfId="24">
+      <calculatedColumnFormula>ISNUMBER(SEARCH("EHDS", G3))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2059,7 +2100,7 @@
       <c r="A11" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="11" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2190,7 +2231,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -2202,8 +2243,8 @@
     <col min="8" max="8" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="191.25" customHeight="1"/>
-    <row r="2" spans="1:8" ht="15">
+    <row r="1" spans="1:9" ht="191.25" customHeight="1"/>
+    <row r="2" spans="1:9" ht="15">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
@@ -2228,145 +2269,176 @@
       <c r="H2" s="18" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" ht="15">
+      <c r="I2" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" ht="15">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="19" t="b">
+        <f t="shared" ref="I3:I9" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" ht="15">
+      <c r="A4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="20" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" ht="29.25">
+      <c r="A5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="2" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" ht="29.25">
+      <c r="A6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" ht="15">
-      <c r="A4" s="2" t="s">
+      <c r="G6" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="I6" s="2" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" ht="15">
+      <c r="A7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="29.25">
-      <c r="A5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" t="s">
-        <v>59</v>
-      </c>
-      <c r="G5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="29.25">
-      <c r="A6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" ht="15">
-      <c r="A7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" t="s">
-        <v>59</v>
-      </c>
       <c r="G7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" ht="20.25" customHeight="1">
+        <v>55</v>
+      </c>
+      <c r="I7" s="2" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="2" customFormat="1" ht="20.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" ht="57.75">
+        <v>55</v>
+      </c>
+      <c r="I8" s="2" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="2" customFormat="1" ht="57.75">
       <c r="A9" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="I9" s="2" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2396,10 +2468,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>42</v>
@@ -2419,13 +2491,13 @@
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" ht="80.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15"/>
@@ -2456,10 +2528,10 @@
     <row r="1" spans="1:7" ht="111" customHeight="1"/>
     <row r="2" spans="1:7" s="16" customFormat="1">
       <c r="A2" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="16" t="s">
         <v>42</v>
@@ -2480,10 +2552,10 @@
     <row r="3" spans="1:7" ht="29.25">
       <c r="A3" s="14"/>
       <c r="B3" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
@@ -2513,7 +2585,7 @@
     <row r="2" spans="1:9">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -2526,16 +2598,16 @@
     <row r="3" spans="1:9">
       <c r="A3" s="3"/>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
@@ -2545,16 +2617,16 @@
     <row r="4" spans="1:9" ht="29.1">
       <c r="A4" s="3"/>
       <c r="B4" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -2563,16 +2635,16 @@
     </row>
     <row r="5" spans="1:9" ht="101.45">
       <c r="B5" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2680,12 +2752,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2896,18 +2970,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2915,5 +2987,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
 </file>
</xml_diff>